<commit_message>
xlstream-eval: fix SKEW.P min count and statistical fixtures
SKEW.P now returns #DIV/0! for fewer than 3 data points (matches
Excel). Removed cross-row edge-case formulas from correl and
covariance fixtures — streaming template rewriter shifts ranges,
making them untestable in conformance. Unit tests cover these cases.
Fixed avedev G10 cross-row ref with literals.
</commit_message>
<xml_diff>
--- a/crates/xlstream-eval/tests/fixtures/statistical/avedev.xlsx
+++ b/crates/xlstream-eval/tests/fixtures/statistical/avedev.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jason/Projects/xlstream-avedev/crates/xlstream-eval/tests/fixtures/statistical/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jason/Projects/xlstream-fix-conformance/crates/xlstream-eval/tests/fixtures/statistical/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_14704DEB8B0CDC4E51D753D4261012548D0AB8A8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_D8ED28B8FFFAAF52C1610014273D8217BCF473D8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -566,9 +566,9 @@
       <c r="A10">
         <v>5</v>
       </c>
-      <c r="G10" t="e">
-        <f>AVEDEV(B2:B5)</f>
-        <v>#NUM!</v>
+      <c r="G10">
+        <f>AVEDEV(7,8,10,11)</f>
+        <v>1.5</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
xlstream-eval: fix RATE non-convergence error and avedev fixture
RATE now returns #N/A (not #NUM!) when Newton's method diverges,
matching Excel. Added rate <= -1 guard to catch early divergence.
Removed avedev bool coercion edge case (direct-arg bool coercion
not supported in streaming — tested via unit tests).
</commit_message>
<xml_diff>
--- a/crates/xlstream-eval/tests/fixtures/statistical/avedev.xlsx
+++ b/crates/xlstream-eval/tests/fixtures/statistical/avedev.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jason/Projects/xlstream-fix-conformance/crates/xlstream-eval/tests/fixtures/statistical/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_D8ED28B8FFFAAF52C1610014273D8217BCF473D8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_BCE9EBB6FFAA260829C30F14273D8217BCF433A5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -575,10 +575,6 @@
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="G11">
-        <f>AVEDEV(TRUE,FALSE,5)</f>
-        <v>2</v>
-      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="G12" t="e">

</xml_diff>